<commit_message>
update resume agent with multi-resume slots and cover letter
</commit_message>
<xml_diff>
--- a/Notes.xlsx
+++ b/Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed1533e5cb63f4dc/Desktop/Claude Projects/resume-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66580341-86CD-4EE3-9B57-152695BD168F}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{040C6991-F8A5-4B16-B518-15AFACDE4FC6}"/>
   <bookViews>
-    <workbookView xWindow="22930" yWindow="1470" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,12 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Features to Add</t>
   </si>
   <si>
     <t>Add LinkedIn Profile</t>
+  </si>
+  <si>
+    <t>Cover letter Input and Tailoring option.</t>
   </si>
 </sst>
 </file>
@@ -83,6 +86,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -348,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -361,6 +368,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>